<commit_message>
test(e2e): add remaining login test cases
- Test Case IDs: TC-LOGIN-003 through TC-LOGIN-011\n- Add login support-link, remember-me, invalid-credential, and masked-password coverage\n- Add forgot-password back-navigation, empty-submit, and field-type coverage\n- Update Test-Cases.xlsx execution tracking\n\nVerified: mvn test -Dheadless=true (10 passed, 1 skipped)\n\nCo-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/KiemTra_1/digishield-e2e/test-cases/Test-Cases.xlsx
+++ b/KiemTra_1/digishield-e2e/test-cases/Test-Cases.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -711,6 +711,699 @@
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Hiển thị đúng các thành phần hỗ trợ đăng nhập</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>navigation-and-ui</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Người dùng đang ở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Không có</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Hiển thị form, liên kết quên mật khẩu và đăng nhập e-mail UTC</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Hiển thị form, liên kết quên mật khẩu và đăng nhập e-mail UTC</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.LoginE2ETest</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>testLoginPageActionsAreAvailable</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Chọn tùy chọn ghi nhớ đăng nhập</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>input-validation</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Người dùng đang ở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>persistent: chưa chọn</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Tùy chọn ghi nhớ đăng nhập được chọn</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Tùy chọn ghi nhớ đăng nhập được chọn</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.LoginE2ETest</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>testRememberMeCanBeSelected</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra liên kết đăng nhập bằng e-mail UTC</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>navigation-and-ui</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>https://accounts.google.com/o/oauth2/auth</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Người dùng đang ở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Không có</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Liên kết hiển thị và trỏ tới luồng OAuth Google</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Liên kết hiển thị và trỏ tới luồng OAuth Google</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.LoginE2ETest</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>testUtcEmailLoginLink</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập với thông tin không hợp lệ</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Người dùng đang ở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>username: automation.invalid@example.com | password: WrongPassword!123</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Không đăng nhập thành công và vẫn ở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Không đăng nhập thành công và vẫn ở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.LoginE2ETest</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>testLoginFailure_InvalidCredentials</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Mật khẩu được hiển thị dưới dạng ký tự ẩn</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>navigation-and-ui</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Người dùng đang ở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Không có</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Trường mật khẩu có type=password</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Trường mật khẩu có type=password</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.LoginE2ETest</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>testPasswordFieldIsMasked</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập thành công với credential do người chạy cung cấp</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>UNTESTED</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Trang sau đăng nhập</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Có tài khoản hợp lệ và truyền -Dusername/-Dpassword</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>username/password qua system properties</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập thành công và rời trang login</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thực thi</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.LoginE2ETest</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>testLoginSuccessWithConfiguredCredentials</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Quay lại trang đăng nhập từ chức năng quên mật khẩu</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Quên mật khẩu</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>navigation-and-ui</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login/GetPass</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Người dùng đã mở trang lấy lại mật khẩu</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Không có</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Điều hướng về login và hiển thị form đăng nhập</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Điều hướng về login và hiển thị form đăng nhập</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.ForgotPasswordE2ETest</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>testBackToLogin</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Submit form lấy lại mật khẩu khi bỏ trống thông tin</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Quên mật khẩu</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>input-validation</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login/GetPass</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login/GetPass</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Người dùng đã mở trang lấy lại mật khẩu</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>captcha/email: trống</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Không rời trang và form tiếp tục hiển thị</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Không rời trang và form tiếp tục hiển thị</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.ForgotPasswordE2ETest</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>testForgotPasswordEmptyFields</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra kiểu dữ liệu các trường lấy lại mật khẩu</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Quên mật khẩu</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>boundary</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login/GetPass</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login/GetPass</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Người dùng đã mở trang lấy lại mật khẩu</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Không có</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Mã bảo mật và email là trường nhập text</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Mã bảo mật và email là trường nhập text</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.ForgotPasswordE2ETest</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>testForgotPasswordFieldTypes</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>JUnit 5 + Selenium WebDriver</t>
         </is>
@@ -742,7 +1435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1020,6 +1713,306 @@
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-003</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Mở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Hiển thị form đăng nhập và các liên kết hỗ trợ</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Hiển thị form đăng nhập và các liên kết hỗ trợ</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-003</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra liên kết quên mật khẩu và e-mail UTC</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Các liên kết hiển thị đúng</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Các liên kết hiển thị đúng</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-004</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Chọn tùy chọn Giữ tôi luôn đăng nhập</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Checkbox persistent chuyển sang trạng thái đã chọn</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Checkbox persistent chuyển sang trạng thái đã chọn</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-005</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra liên kết Đăng nhập bằng e-mail UTC</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Href trỏ tới accounts.google.com OAuth</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Href trỏ tới accounts.google.com OAuth</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-006</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Nhập username/password không hợp lệ và nhấn Đăng nhập</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Không đăng nhập thành công, vẫn ở trang login</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Không đăng nhập thành công, vẫn ở trang login</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-007</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra thuộc tính trường Mật khẩu</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Trường có type=password</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Trường có type=password</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-008</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Nhập credential qua system properties và nhấn Đăng nhập</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển khỏi trang login khi credential hợp lệ</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thực thi</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>UNTESTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-009</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Mở trang lấy lại mật khẩu và chọn Trở lại đăng nhập</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Điều hướng về /Login</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Điều hướng về /Login</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-010</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Để trống Mã bảo mật và Địa chỉ Email rồi chọn Cập nhật</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Vẫn ở /Login/GetPass và form hiển thị</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Vẫn ở /Login/GetPass và form hiển thị</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-011</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra type của Mã bảo mật và Địa chỉ Email</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Cả hai trường có type=text</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Cả hai trường có type=text</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>

<commit_message>
test(e2e): add five login coverage cases
- Test Case IDs: TC-LOGIN-012 through TC-LOGIN-016\n- Cover login page title, retained form values, remember-me idempotency, support links, and captcha image\n- Update Test-Cases.xlsx execution tracking\n\nVerified: mvn clean test -Dheadless=true -Dtest=LoginE2ETest,ForgotPasswordE2ETest (16 tests, 0 failures, 1 skipped)\n\nCo-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/KiemTra_1/digishield-e2e/test-cases/Test-Cases.xlsx
+++ b/KiemTra_1/digishield-e2e/test-cases/Test-Cases.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1404,6 +1404,391 @@
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra tiêu đề trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>navigation-and-ui</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Người dùng đang ở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Không có</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>URL và tiêu đề là Đăng nhập</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>URL và tiêu đề đúng</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.LoginE2ETest</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>testLoginPageTitle</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Giá trị nhập vào được giữ trong form đăng nhập</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>input-validation</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Người dùng đang ở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>username: test.user@example.com | password: TestPassword!123</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Form giữ đúng username và password vừa nhập</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Giá trị được giữ đúng</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.LoginE2ETest</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>testLoginFormRetainsEnteredValues</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Thao tác chọn ghi nhớ đăng nhập có tính idempotent</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>input-validation</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Người dùng đang ở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Thao tác chọn ghi nhớ đăng nhập hai lần</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Checkbox vẫn ở trạng thái đã chọn</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Checkbox vẫn được chọn</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.LoginE2ETest</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>testRememberMeSelectionIsIdempotent</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra liên kết trợ giúp và phản hồi</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Đăng nhập</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>navigation-and-ui</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>http://hotrokythuat.utc.edu.vn/ và mailto:hotrokythuat@utc.edu.vn</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Người dùng đang ở trang đăng nhập</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Không có</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Hiển thị đúng liên kết Trung tâm trợ giúp và Ý kiến phản hồi</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Các liên kết đúng</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.LoginE2ETest</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>testSupportLinks</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>JUnit 5 + Selenium WebDriver</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra ảnh mã bảo mật trên trang lấy lại mật khẩu</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Quên mật khẩu</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>navigation-and-ui</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login/GetPass</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>https://vanphongdientu.utc.edu.vn/Login/GetPass</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Người dùng đã mở trang lấy lại mật khẩu</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Không có</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Ảnh captcha hiển thị và dùng endpoint /login/index/captcha</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Ảnh captcha hiển thị đúng</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>com.digishield.e2e.tests.ForgotPasswordE2ETest</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>testCaptchaImage</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
         <is>
           <t>JUnit 5 + Selenium WebDriver</t>
         </is>
@@ -1435,7 +1820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2013,6 +2398,156 @@
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-012</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Mở trang đăng nhập và kiểm tra URL, tiêu đề</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>URL đúng và tiêu đề là Đăng nhập</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>URL và tiêu đề đúng</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-013</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Nhập username và password</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Các giá trị nhập được giữ trong form</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Giá trị được giữ đúng</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-014</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Chọn ghi nhớ đăng nhập hai lần</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Checkbox vẫn được chọn</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Checkbox vẫn được chọn</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-015</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm tra liên kết Trung tâm trợ giúp và Ý kiến phản hồi</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Href đúng với website trợ giúp và email phản hồi</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Các liên kết đúng</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TC-LOGIN-016</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Mở trang lấy lại mật khẩu và kiểm tra ảnh captcha</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Ảnh captcha hiển thị từ endpoint /login/index/captcha</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Ảnh captcha hiển thị đúng</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>